<commit_message>
feat: Catch up 02-25 session work — call list, VetsBoats report, SEO schema, sample report, nonprofit one-pager
Includes call list improvements, VetsBoats consolidated master report,
SEO schema enhancement prompts/reports, sample report update for Netlify,
and nonprofit one-pager (PDF in gitignored 6. Business/ folder).

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ToDo.xlsx
+++ b/ToDo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aleckleinman/Documents/TheGrantScout/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BA2FAE4-9A7F-C94B-934B-E3F963016C9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8DEAD82-EEE0-3245-ABD0-ACC9078E84C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19280" yWindow="500" windowWidth="18960" windowHeight="19200" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="140" yWindow="680" windowWidth="18960" windowHeight="19220" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="9" r:id="rId1"/>
@@ -22,7 +22,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Beta Leads'!$B$3:$N$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To Do'!$B$2:$H$172</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To Do'!$B$2:$H$179</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="290">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="301">
   <si>
     <t>Task</t>
   </si>
@@ -931,6 +931,39 @@
   </si>
   <si>
     <t>Meeting Scheduled</t>
+  </si>
+  <si>
+    <t>Linkedin posts on Fridays</t>
+  </si>
+  <si>
+    <t>update TGS data dictionary</t>
+  </si>
+  <si>
+    <t>Analyze VB report process</t>
+  </si>
+  <si>
+    <t>Research CNE adhacent companies</t>
+  </si>
+  <si>
+    <t>Email accountability my KPI goals for the week (and my new process)</t>
+  </si>
+  <si>
+    <t>Open the leads excel sheet and see who to follow up with? (afternoon activity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Learn about what kind of nonprofits we can work with now that we have section I data (public charities) </t>
+  </si>
+  <si>
+    <t>How does the I data impact our reports flow?</t>
+  </si>
+  <si>
+    <t>How much time did we save Matt looking through websites to find out eligibility - add that to the website</t>
+  </si>
+  <si>
+    <t>Put a more current example report on the website</t>
+  </si>
+  <si>
+    <t>Make Matts March Report</t>
   </si>
 </sst>
 </file>
@@ -1286,7 +1319,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1459,12 +1492,225 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="13">
+  <dxfs count="37">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9966"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF7FDAA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF99CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9966"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFB7C3FD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF99CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFABE0FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF99CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFB7C3FD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF99CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9966"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFB7C3FD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF99CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9966"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1514,57 +1760,19 @@
         </patternFill>
       </fill>
     </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFB7C3FD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF99CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF9966"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFC6C7FF"/>
+      <color rgb="FF9999FF"/>
+      <color rgb="FFABE0FF"/>
+      <color rgb="FFBAE9EF"/>
+      <color rgb="FFF7FDAA"/>
       <color rgb="FFB7C3FD"/>
       <color rgb="FFCCCCFF"/>
       <color rgb="FFFFCCFF"/>
       <color rgb="FFFF9966"/>
-      <color rgb="FF9999FF"/>
       <color rgb="FFFF99CC"/>
     </mruColors>
   </colors>
@@ -2096,7 +2304,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40A518F1-E8D1-4EDA-B8FC-EAEFD9F39116}">
-  <dimension ref="B1:S172"/>
+  <dimension ref="B1:S179"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="23.5" style="66" customWidth="1"/>
@@ -2154,7 +2362,7 @@
         <v>45992</v>
       </c>
       <c r="C3" s="69" t="str">
-        <f t="shared" ref="C3:C11" si="0">TEXT(B3, "dddd")</f>
+        <f>TEXT(B3, "dddd")</f>
         <v>Monday</v>
       </c>
       <c r="D3" s="70">
@@ -2187,7 +2395,7 @@
         <v>45992</v>
       </c>
       <c r="C4" s="14" t="str">
-        <f t="shared" si="0"/>
+        <f>TEXT(B4, "dddd")</f>
         <v>Monday</v>
       </c>
       <c r="D4" s="15">
@@ -2220,7 +2428,7 @@
         <v>45992</v>
       </c>
       <c r="C5" s="14" t="str">
-        <f t="shared" si="0"/>
+        <f>TEXT(B5, "dddd")</f>
         <v>Monday</v>
       </c>
       <c r="D5" s="15">
@@ -2253,7 +2461,7 @@
         <v>45992</v>
       </c>
       <c r="C6" s="14" t="str">
-        <f t="shared" si="0"/>
+        <f>TEXT(B6, "dddd")</f>
         <v>Monday</v>
       </c>
       <c r="D6" s="15">
@@ -2286,7 +2494,7 @@
         <v>45992</v>
       </c>
       <c r="C7" s="14" t="str">
-        <f t="shared" si="0"/>
+        <f>TEXT(B7, "dddd")</f>
         <v>Monday</v>
       </c>
       <c r="D7" s="15">
@@ -2319,7 +2527,7 @@
         <v>45992</v>
       </c>
       <c r="C8" s="14" t="str">
-        <f t="shared" si="0"/>
+        <f>TEXT(B8, "dddd")</f>
         <v>Monday</v>
       </c>
       <c r="D8" s="15">
@@ -2352,7 +2560,7 @@
         <v>45992</v>
       </c>
       <c r="C9" s="14" t="str">
-        <f t="shared" si="0"/>
+        <f>TEXT(B9, "dddd")</f>
         <v>Monday</v>
       </c>
       <c r="D9" s="15">
@@ -2385,7 +2593,7 @@
         <v>45992</v>
       </c>
       <c r="C10" s="14" t="str">
-        <f t="shared" si="0"/>
+        <f>TEXT(B10, "dddd")</f>
         <v>Monday</v>
       </c>
       <c r="D10" s="15">
@@ -2418,7 +2626,7 @@
         <v>45992</v>
       </c>
       <c r="C11" s="14" t="str">
-        <f t="shared" si="0"/>
+        <f>TEXT(B11, "dddd")</f>
         <v>Monday</v>
       </c>
       <c r="D11" s="15">
@@ -2451,7 +2659,7 @@
         <v>45992</v>
       </c>
       <c r="C12" s="15" t="str">
-        <f t="shared" ref="C12:C43" si="1">IF(ISBLANK(B12),"",TEXT(B12, "dddd"))</f>
+        <f>IF(ISBLANK(B12),"",TEXT(B12, "dddd"))</f>
         <v>Monday</v>
       </c>
       <c r="D12" s="15">
@@ -2484,7 +2692,7 @@
         <v>45994</v>
       </c>
       <c r="C13" s="15" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISBLANK(B13),"",TEXT(B13, "dddd"))</f>
         <v>Wednesday</v>
       </c>
       <c r="D13" s="15">
@@ -2517,7 +2725,7 @@
         <v>45994</v>
       </c>
       <c r="C14" s="15" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISBLANK(B14),"",TEXT(B14, "dddd"))</f>
         <v>Wednesday</v>
       </c>
       <c r="D14" s="15">
@@ -2550,7 +2758,7 @@
         <v>45994</v>
       </c>
       <c r="C15" s="15" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISBLANK(B15),"",TEXT(B15, "dddd"))</f>
         <v>Wednesday</v>
       </c>
       <c r="D15" s="38">
@@ -2583,7 +2791,7 @@
         <v>45994</v>
       </c>
       <c r="C16" s="15" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISBLANK(B16),"",TEXT(B16, "dddd"))</f>
         <v>Wednesday</v>
       </c>
       <c r="D16" s="15">
@@ -2616,7 +2824,7 @@
         <v>45994</v>
       </c>
       <c r="C17" s="15" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISBLANK(B17),"",TEXT(B17, "dddd"))</f>
         <v>Wednesday</v>
       </c>
       <c r="D17" s="15">
@@ -2649,7 +2857,7 @@
         <v>45994</v>
       </c>
       <c r="C18" s="15" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISBLANK(B18),"",TEXT(B18, "dddd"))</f>
         <v>Wednesday</v>
       </c>
       <c r="D18" s="15">
@@ -2682,7 +2890,7 @@
         <v>45994</v>
       </c>
       <c r="C19" s="15" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISBLANK(B19),"",TEXT(B19, "dddd"))</f>
         <v>Wednesday</v>
       </c>
       <c r="D19" s="15">
@@ -2715,7 +2923,7 @@
         <v>45994</v>
       </c>
       <c r="C20" s="15" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISBLANK(B20),"",TEXT(B20, "dddd"))</f>
         <v>Wednesday</v>
       </c>
       <c r="D20" s="15">
@@ -2748,7 +2956,7 @@
         <v>45995</v>
       </c>
       <c r="C21" s="15" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISBLANK(B21),"",TEXT(B21, "dddd"))</f>
         <v>Thursday</v>
       </c>
       <c r="D21" s="15">
@@ -2781,7 +2989,7 @@
         <v>45995</v>
       </c>
       <c r="C22" s="15" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISBLANK(B22),"",TEXT(B22, "dddd"))</f>
         <v>Thursday</v>
       </c>
       <c r="D22" s="15">
@@ -2814,7 +3022,7 @@
         <v>45995</v>
       </c>
       <c r="C23" s="15" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISBLANK(B23),"",TEXT(B23, "dddd"))</f>
         <v>Thursday</v>
       </c>
       <c r="D23" s="15">
@@ -2847,7 +3055,7 @@
         <v>45995</v>
       </c>
       <c r="C24" s="15" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISBLANK(B24),"",TEXT(B24, "dddd"))</f>
         <v>Thursday</v>
       </c>
       <c r="D24" s="15">
@@ -2880,7 +3088,7 @@
         <v>45995</v>
       </c>
       <c r="C25" s="15" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISBLANK(B25),"",TEXT(B25, "dddd"))</f>
         <v>Thursday</v>
       </c>
       <c r="D25" s="15">
@@ -2913,7 +3121,7 @@
         <v>45995</v>
       </c>
       <c r="C26" s="15" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISBLANK(B26),"",TEXT(B26, "dddd"))</f>
         <v>Thursday</v>
       </c>
       <c r="D26" s="15">
@@ -2946,7 +3154,7 @@
         <v>45995</v>
       </c>
       <c r="C27" s="15" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISBLANK(B27),"",TEXT(B27, "dddd"))</f>
         <v>Thursday</v>
       </c>
       <c r="D27" s="15"/>
@@ -2975,7 +3183,7 @@
         <v>45996</v>
       </c>
       <c r="C28" s="15" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISBLANK(B28),"",TEXT(B28, "dddd"))</f>
         <v>Friday</v>
       </c>
       <c r="D28" s="15">
@@ -3008,7 +3216,7 @@
         <v>45996</v>
       </c>
       <c r="C29" s="15" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISBLANK(B29),"",TEXT(B29, "dddd"))</f>
         <v>Friday</v>
       </c>
       <c r="D29" s="15">
@@ -3041,7 +3249,7 @@
         <v>45996</v>
       </c>
       <c r="C30" s="15" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISBLANK(B30),"",TEXT(B30, "dddd"))</f>
         <v>Friday</v>
       </c>
       <c r="D30" s="15">
@@ -3074,7 +3282,7 @@
         <v>45996</v>
       </c>
       <c r="C31" s="15" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISBLANK(B31),"",TEXT(B31, "dddd"))</f>
         <v>Friday</v>
       </c>
       <c r="D31" s="15">
@@ -3107,7 +3315,7 @@
         <v>45996</v>
       </c>
       <c r="C32" s="15" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISBLANK(B32),"",TEXT(B32, "dddd"))</f>
         <v>Friday</v>
       </c>
       <c r="D32" s="15"/>
@@ -3138,7 +3346,7 @@
         <v>45999</v>
       </c>
       <c r="C33" s="15" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISBLANK(B33),"",TEXT(B33, "dddd"))</f>
         <v>Monday</v>
       </c>
       <c r="D33" s="15">
@@ -3156,7 +3364,7 @@
         <v>45999</v>
       </c>
       <c r="C34" s="15" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISBLANK(B34),"",TEXT(B34, "dddd"))</f>
         <v>Monday</v>
       </c>
       <c r="D34" s="15">
@@ -3174,7 +3382,7 @@
         <v>45999</v>
       </c>
       <c r="C35" s="15" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISBLANK(B35),"",TEXT(B35, "dddd"))</f>
         <v>Monday</v>
       </c>
       <c r="D35" s="15">
@@ -3192,7 +3400,7 @@
         <v>45999</v>
       </c>
       <c r="C36" s="15" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISBLANK(B36),"",TEXT(B36, "dddd"))</f>
         <v>Monday</v>
       </c>
       <c r="D36" s="15">
@@ -3210,7 +3418,7 @@
         <v>46000</v>
       </c>
       <c r="C37" s="15" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISBLANK(B37),"",TEXT(B37, "dddd"))</f>
         <v>Tuesday</v>
       </c>
       <c r="D37" s="15"/>
@@ -3230,7 +3438,7 @@
         <v>46001</v>
       </c>
       <c r="C38" s="15" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISBLANK(B38),"",TEXT(B38, "dddd"))</f>
         <v>Wednesday</v>
       </c>
       <c r="D38" s="15">
@@ -3252,7 +3460,7 @@
         <v>46001</v>
       </c>
       <c r="C39" s="15" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISBLANK(B39),"",TEXT(B39, "dddd"))</f>
         <v>Wednesday</v>
       </c>
       <c r="D39" s="15">
@@ -3274,7 +3482,7 @@
         <v>46001</v>
       </c>
       <c r="C40" s="15" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISBLANK(B40),"",TEXT(B40, "dddd"))</f>
         <v>Wednesday</v>
       </c>
       <c r="D40" s="15">
@@ -3296,7 +3504,7 @@
         <v>46001</v>
       </c>
       <c r="C41" s="15" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISBLANK(B41),"",TEXT(B41, "dddd"))</f>
         <v>Wednesday</v>
       </c>
       <c r="D41" s="15">
@@ -3318,7 +3526,7 @@
         <v>46001</v>
       </c>
       <c r="C42" s="15" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISBLANK(B42),"",TEXT(B42, "dddd"))</f>
         <v>Wednesday</v>
       </c>
       <c r="D42" s="15">
@@ -3340,7 +3548,7 @@
         <v>46001</v>
       </c>
       <c r="C43" s="15" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(ISBLANK(B43),"",TEXT(B43, "dddd"))</f>
         <v>Wednesday</v>
       </c>
       <c r="D43" s="15">
@@ -3362,7 +3570,7 @@
         <v>46001</v>
       </c>
       <c r="C44" s="15" t="str">
-        <f t="shared" ref="C44:C75" si="2">IF(ISBLANK(B44),"",TEXT(B44, "dddd"))</f>
+        <f>IF(ISBLANK(B44),"",TEXT(B44, "dddd"))</f>
         <v>Wednesday</v>
       </c>
       <c r="D44" s="15">
@@ -3380,7 +3588,7 @@
         <v>46001</v>
       </c>
       <c r="C45" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ISBLANK(B45),"",TEXT(B45, "dddd"))</f>
         <v>Wednesday</v>
       </c>
       <c r="D45" s="15">
@@ -3400,7 +3608,7 @@
         <v>46001</v>
       </c>
       <c r="C46" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ISBLANK(B46),"",TEXT(B46, "dddd"))</f>
         <v>Wednesday</v>
       </c>
       <c r="D46" s="15">
@@ -3420,7 +3628,7 @@
         <v>46001</v>
       </c>
       <c r="C47" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ISBLANK(B47),"",TEXT(B47, "dddd"))</f>
         <v>Wednesday</v>
       </c>
       <c r="D47" s="15">
@@ -3442,7 +3650,7 @@
         <v>46002</v>
       </c>
       <c r="C48" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ISBLANK(B48),"",TEXT(B48, "dddd"))</f>
         <v>Thursday</v>
       </c>
       <c r="D48" s="15">
@@ -3462,7 +3670,7 @@
         <v>46003</v>
       </c>
       <c r="C49" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ISBLANK(B49),"",TEXT(B49, "dddd"))</f>
         <v>Friday</v>
       </c>
       <c r="D49" s="15">
@@ -3484,7 +3692,7 @@
         <v>46006</v>
       </c>
       <c r="C50" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ISBLANK(B50),"",TEXT(B50, "dddd"))</f>
         <v>Monday</v>
       </c>
       <c r="D50" s="15">
@@ -3506,7 +3714,7 @@
         <v>46006</v>
       </c>
       <c r="C51" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ISBLANK(B51),"",TEXT(B51, "dddd"))</f>
         <v>Monday</v>
       </c>
       <c r="D51" s="15">
@@ -3528,7 +3736,7 @@
         <v>46006</v>
       </c>
       <c r="C52" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ISBLANK(B52),"",TEXT(B52, "dddd"))</f>
         <v>Monday</v>
       </c>
       <c r="D52" s="15">
@@ -3550,7 +3758,7 @@
         <v>46006</v>
       </c>
       <c r="C53" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ISBLANK(B53),"",TEXT(B53, "dddd"))</f>
         <v>Monday</v>
       </c>
       <c r="D53" s="15">
@@ -3572,7 +3780,7 @@
         <v>46006</v>
       </c>
       <c r="C54" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ISBLANK(B54),"",TEXT(B54, "dddd"))</f>
         <v>Monday</v>
       </c>
       <c r="D54" s="15">
@@ -3594,7 +3802,7 @@
         <v>46006</v>
       </c>
       <c r="C55" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ISBLANK(B55),"",TEXT(B55, "dddd"))</f>
         <v>Monday</v>
       </c>
       <c r="D55" s="15">
@@ -3616,7 +3824,7 @@
         <v>46006</v>
       </c>
       <c r="C56" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ISBLANK(B56),"",TEXT(B56, "dddd"))</f>
         <v>Monday</v>
       </c>
       <c r="D56" s="15">
@@ -3638,7 +3846,7 @@
         <v>46006</v>
       </c>
       <c r="C57" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ISBLANK(B57),"",TEXT(B57, "dddd"))</f>
         <v>Monday</v>
       </c>
       <c r="D57" s="15">
@@ -3660,7 +3868,7 @@
         <v>46006</v>
       </c>
       <c r="C58" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ISBLANK(B58),"",TEXT(B58, "dddd"))</f>
         <v>Monday</v>
       </c>
       <c r="D58" s="15">
@@ -3682,7 +3890,7 @@
         <v>46006</v>
       </c>
       <c r="C59" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ISBLANK(B59),"",TEXT(B59, "dddd"))</f>
         <v>Monday</v>
       </c>
       <c r="D59" s="15">
@@ -3704,7 +3912,7 @@
         <v>46006</v>
       </c>
       <c r="C60" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ISBLANK(B60),"",TEXT(B60, "dddd"))</f>
         <v>Monday</v>
       </c>
       <c r="D60" s="15">
@@ -3726,7 +3934,7 @@
         <v>46007</v>
       </c>
       <c r="C61" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ISBLANK(B61),"",TEXT(B61, "dddd"))</f>
         <v>Tuesday</v>
       </c>
       <c r="D61" s="15">
@@ -3748,7 +3956,7 @@
         <v>46007</v>
       </c>
       <c r="C62" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ISBLANK(B62),"",TEXT(B62, "dddd"))</f>
         <v>Tuesday</v>
       </c>
       <c r="D62" s="15">
@@ -3770,7 +3978,7 @@
         <v>46007</v>
       </c>
       <c r="C63" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ISBLANK(B63),"",TEXT(B63, "dddd"))</f>
         <v>Tuesday</v>
       </c>
       <c r="D63" s="15">
@@ -3792,7 +4000,7 @@
         <v>46007</v>
       </c>
       <c r="C64" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ISBLANK(B64),"",TEXT(B64, "dddd"))</f>
         <v>Tuesday</v>
       </c>
       <c r="D64" s="15">
@@ -3814,7 +4022,7 @@
         <v>46008</v>
       </c>
       <c r="C65" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ISBLANK(B65),"",TEXT(B65, "dddd"))</f>
         <v>Wednesday</v>
       </c>
       <c r="D65" s="15">
@@ -3834,7 +4042,7 @@
         <v>46008</v>
       </c>
       <c r="C66" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ISBLANK(B66),"",TEXT(B66, "dddd"))</f>
         <v>Wednesday</v>
       </c>
       <c r="D66" s="15">
@@ -3854,7 +4062,7 @@
         <v>46008</v>
       </c>
       <c r="C67" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ISBLANK(B67),"",TEXT(B67, "dddd"))</f>
         <v>Wednesday</v>
       </c>
       <c r="D67" s="15">
@@ -3872,7 +4080,7 @@
         <v>46008</v>
       </c>
       <c r="C68" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ISBLANK(B68),"",TEXT(B68, "dddd"))</f>
         <v>Wednesday</v>
       </c>
       <c r="D68" s="15">
@@ -3892,7 +4100,7 @@
         <v>46009</v>
       </c>
       <c r="C69" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ISBLANK(B69),"",TEXT(B69, "dddd"))</f>
         <v>Thursday</v>
       </c>
       <c r="D69" s="15">
@@ -3912,7 +4120,7 @@
         <v>46009</v>
       </c>
       <c r="C70" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ISBLANK(B70),"",TEXT(B70, "dddd"))</f>
         <v>Thursday</v>
       </c>
       <c r="D70" s="15"/>
@@ -3930,7 +4138,7 @@
         <v>46015</v>
       </c>
       <c r="C71" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ISBLANK(B71),"",TEXT(B71, "dddd"))</f>
         <v>Wednesday</v>
       </c>
       <c r="D71" s="15">
@@ -3950,7 +4158,7 @@
         <v>46015</v>
       </c>
       <c r="C72" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ISBLANK(B72),"",TEXT(B72, "dddd"))</f>
         <v>Wednesday</v>
       </c>
       <c r="D72" s="15">
@@ -3970,7 +4178,7 @@
         <v>46015</v>
       </c>
       <c r="C73" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ISBLANK(B73),"",TEXT(B73, "dddd"))</f>
         <v>Wednesday</v>
       </c>
       <c r="D73" s="15"/>
@@ -3988,7 +4196,7 @@
         <v>46015</v>
       </c>
       <c r="C74" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ISBLANK(B74),"",TEXT(B74, "dddd"))</f>
         <v>Wednesday</v>
       </c>
       <c r="D74" s="15"/>
@@ -4006,7 +4214,7 @@
         <v>46015</v>
       </c>
       <c r="C75" s="15" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(ISBLANK(B75),"",TEXT(B75, "dddd"))</f>
         <v>Wednesday</v>
       </c>
       <c r="D75" s="15"/>
@@ -4024,7 +4232,7 @@
         <v>46022</v>
       </c>
       <c r="C76" s="15" t="str">
-        <f t="shared" ref="C76:C107" si="3">IF(ISBLANK(B76),"",TEXT(B76, "dddd"))</f>
+        <f>IF(ISBLANK(B76),"",TEXT(B76, "dddd"))</f>
         <v>Wednesday</v>
       </c>
       <c r="D76" s="15"/>
@@ -4042,7 +4250,7 @@
         <v>46022</v>
       </c>
       <c r="C77" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ISBLANK(B77),"",TEXT(B77, "dddd"))</f>
         <v>Wednesday</v>
       </c>
       <c r="D77" s="15"/>
@@ -4060,7 +4268,7 @@
         <v>46022</v>
       </c>
       <c r="C78" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ISBLANK(B78),"",TEXT(B78, "dddd"))</f>
         <v>Wednesday</v>
       </c>
       <c r="D78" s="15"/>
@@ -4078,7 +4286,7 @@
         <v>46024</v>
       </c>
       <c r="C79" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ISBLANK(B79),"",TEXT(B79, "dddd"))</f>
         <v>Friday</v>
       </c>
       <c r="D79" s="15">
@@ -4098,7 +4306,7 @@
         <v>46024</v>
       </c>
       <c r="C80" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ISBLANK(B80),"",TEXT(B80, "dddd"))</f>
         <v>Friday</v>
       </c>
       <c r="D80" s="15">
@@ -4118,7 +4326,7 @@
         <v>46024</v>
       </c>
       <c r="C81" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ISBLANK(B81),"",TEXT(B81, "dddd"))</f>
         <v>Friday</v>
       </c>
       <c r="D81" s="15">
@@ -4138,7 +4346,7 @@
         <v>46024</v>
       </c>
       <c r="C82" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ISBLANK(B82),"",TEXT(B82, "dddd"))</f>
         <v>Friday</v>
       </c>
       <c r="D82" s="15">
@@ -4158,7 +4366,7 @@
         <v>46024</v>
       </c>
       <c r="C83" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ISBLANK(B83),"",TEXT(B83, "dddd"))</f>
         <v>Friday</v>
       </c>
       <c r="D83" s="15">
@@ -4178,7 +4386,7 @@
         <v>46024</v>
       </c>
       <c r="C84" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ISBLANK(B84),"",TEXT(B84, "dddd"))</f>
         <v>Friday</v>
       </c>
       <c r="D84" s="15">
@@ -4198,7 +4406,7 @@
         <v>46024</v>
       </c>
       <c r="C85" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ISBLANK(B85),"",TEXT(B85, "dddd"))</f>
         <v>Friday</v>
       </c>
       <c r="D85" s="15">
@@ -4218,7 +4426,7 @@
         <v>46024</v>
       </c>
       <c r="C86" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ISBLANK(B86),"",TEXT(B86, "dddd"))</f>
         <v>Friday</v>
       </c>
       <c r="D86" s="15">
@@ -4236,7 +4444,7 @@
         <v>46024</v>
       </c>
       <c r="C87" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ISBLANK(B87),"",TEXT(B87, "dddd"))</f>
         <v>Friday</v>
       </c>
       <c r="D87" s="15">
@@ -4256,7 +4464,7 @@
         <v>46024</v>
       </c>
       <c r="C88" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ISBLANK(B88),"",TEXT(B88, "dddd"))</f>
         <v>Friday</v>
       </c>
       <c r="D88" s="15">
@@ -4274,7 +4482,7 @@
         <v>46024</v>
       </c>
       <c r="C89" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ISBLANK(B89),"",TEXT(B89, "dddd"))</f>
         <v>Friday</v>
       </c>
       <c r="D89" s="15">
@@ -4294,7 +4502,7 @@
         <v>46024</v>
       </c>
       <c r="C90" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ISBLANK(B90),"",TEXT(B90, "dddd"))</f>
         <v>Friday</v>
       </c>
       <c r="D90" s="15">
@@ -4314,7 +4522,7 @@
         <v>46024</v>
       </c>
       <c r="C91" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ISBLANK(B91),"",TEXT(B91, "dddd"))</f>
         <v>Friday</v>
       </c>
       <c r="D91" s="15">
@@ -4334,7 +4542,7 @@
         <v>46024</v>
       </c>
       <c r="C92" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ISBLANK(B92),"",TEXT(B92, "dddd"))</f>
         <v>Friday</v>
       </c>
       <c r="D92" s="15">
@@ -4354,7 +4562,7 @@
         <v>46024</v>
       </c>
       <c r="C93" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ISBLANK(B93),"",TEXT(B93, "dddd"))</f>
         <v>Friday</v>
       </c>
       <c r="D93" s="15">
@@ -4374,7 +4582,7 @@
         <v>46024</v>
       </c>
       <c r="C94" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ISBLANK(B94),"",TEXT(B94, "dddd"))</f>
         <v>Friday</v>
       </c>
       <c r="D94" s="15">
@@ -4394,7 +4602,7 @@
         <v>46024</v>
       </c>
       <c r="C95" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ISBLANK(B95),"",TEXT(B95, "dddd"))</f>
         <v>Friday</v>
       </c>
       <c r="D95" s="15">
@@ -4414,7 +4622,7 @@
         <v>46024</v>
       </c>
       <c r="C96" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ISBLANK(B96),"",TEXT(B96, "dddd"))</f>
         <v>Friday</v>
       </c>
       <c r="D96" s="15">
@@ -4434,7 +4642,7 @@
         <v>46024</v>
       </c>
       <c r="C97" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ISBLANK(B97),"",TEXT(B97, "dddd"))</f>
         <v>Friday</v>
       </c>
       <c r="D97" s="15">
@@ -4452,7 +4660,7 @@
         <v>46024</v>
       </c>
       <c r="C98" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ISBLANK(B98),"",TEXT(B98, "dddd"))</f>
         <v>Friday</v>
       </c>
       <c r="D98" s="15">
@@ -4470,7 +4678,7 @@
         <v>46024</v>
       </c>
       <c r="C99" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ISBLANK(B99),"",TEXT(B99, "dddd"))</f>
         <v>Friday</v>
       </c>
       <c r="D99" s="15">
@@ -4488,7 +4696,7 @@
         <v>46027</v>
       </c>
       <c r="C100" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ISBLANK(B100),"",TEXT(B100, "dddd"))</f>
         <v>Monday</v>
       </c>
       <c r="D100" s="15"/>
@@ -4506,7 +4714,7 @@
         <v>46028</v>
       </c>
       <c r="C101" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ISBLANK(B101),"",TEXT(B101, "dddd"))</f>
         <v>Tuesday</v>
       </c>
       <c r="D101" s="15"/>
@@ -4524,7 +4732,7 @@
         <v>46028</v>
       </c>
       <c r="C102" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ISBLANK(B102),"",TEXT(B102, "dddd"))</f>
         <v>Tuesday</v>
       </c>
       <c r="D102" s="15"/>
@@ -4540,7 +4748,7 @@
         <v>46028</v>
       </c>
       <c r="C103" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ISBLANK(B103),"",TEXT(B103, "dddd"))</f>
         <v>Tuesday</v>
       </c>
       <c r="D103" s="15"/>
@@ -4556,7 +4764,7 @@
         <v>46030</v>
       </c>
       <c r="C104" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ISBLANK(B104),"",TEXT(B104, "dddd"))</f>
         <v>Thursday</v>
       </c>
       <c r="D104" s="15"/>
@@ -4576,7 +4784,7 @@
         <v>46030</v>
       </c>
       <c r="C105" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ISBLANK(B105),"",TEXT(B105, "dddd"))</f>
         <v>Thursday</v>
       </c>
       <c r="D105" s="15"/>
@@ -4596,7 +4804,7 @@
         <v>46034</v>
       </c>
       <c r="C106" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ISBLANK(B106),"",TEXT(B106, "dddd"))</f>
         <v>Monday</v>
       </c>
       <c r="D106" s="15"/>
@@ -4616,7 +4824,7 @@
         <v>46035</v>
       </c>
       <c r="C107" s="15" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(ISBLANK(B107),"",TEXT(B107, "dddd"))</f>
         <v>Tuesday</v>
       </c>
       <c r="D107" s="15">
@@ -4636,7 +4844,7 @@
         <v>46035</v>
       </c>
       <c r="C108" s="15" t="str">
-        <f t="shared" ref="C108:C139" si="4">IF(ISBLANK(B108),"",TEXT(B108, "dddd"))</f>
+        <f>IF(ISBLANK(B108),"",TEXT(B108, "dddd"))</f>
         <v>Tuesday</v>
       </c>
       <c r="D108" s="15">
@@ -4656,7 +4864,7 @@
         <v>46036</v>
       </c>
       <c r="C109" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f>IF(ISBLANK(B109),"",TEXT(B109, "dddd"))</f>
         <v>Wednesday</v>
       </c>
       <c r="D109" s="15"/>
@@ -4674,7 +4882,7 @@
         <v>46036</v>
       </c>
       <c r="C110" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f>IF(ISBLANK(B110),"",TEXT(B110, "dddd"))</f>
         <v>Wednesday</v>
       </c>
       <c r="D110" s="15"/>
@@ -4692,7 +4900,7 @@
         <v>46036</v>
       </c>
       <c r="C111" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f>IF(ISBLANK(B111),"",TEXT(B111, "dddd"))</f>
         <v>Wednesday</v>
       </c>
       <c r="D111" s="15"/>
@@ -4710,7 +4918,7 @@
         <v>46036</v>
       </c>
       <c r="C112" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f>IF(ISBLANK(B112),"",TEXT(B112, "dddd"))</f>
         <v>Wednesday</v>
       </c>
       <c r="D112" s="15"/>
@@ -4728,7 +4936,7 @@
         <v>46037</v>
       </c>
       <c r="C113" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f>IF(ISBLANK(B113),"",TEXT(B113, "dddd"))</f>
         <v>Thursday</v>
       </c>
       <c r="D113" s="15"/>
@@ -4746,7 +4954,7 @@
         <v>46038</v>
       </c>
       <c r="C114" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f>IF(ISBLANK(B114),"",TEXT(B114, "dddd"))</f>
         <v>Friday</v>
       </c>
       <c r="D114" s="15">
@@ -4768,7 +4976,7 @@
         <v>46038</v>
       </c>
       <c r="C115" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f>IF(ISBLANK(B115),"",TEXT(B115, "dddd"))</f>
         <v>Friday</v>
       </c>
       <c r="D115" s="15">
@@ -4790,7 +4998,7 @@
         <v>46038</v>
       </c>
       <c r="C116" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f>IF(ISBLANK(B116),"",TEXT(B116, "dddd"))</f>
         <v>Friday</v>
       </c>
       <c r="D116" s="15">
@@ -4812,7 +5020,7 @@
         <v>46038</v>
       </c>
       <c r="C117" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f>IF(ISBLANK(B117),"",TEXT(B117, "dddd"))</f>
         <v>Friday</v>
       </c>
       <c r="D117" s="15"/>
@@ -4826,7 +5034,7 @@
         <v>46042</v>
       </c>
       <c r="C118" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f>IF(ISBLANK(B118),"",TEXT(B118, "dddd"))</f>
         <v>Tuesday</v>
       </c>
       <c r="D118" s="15"/>
@@ -4846,7 +5054,7 @@
         <v>46042</v>
       </c>
       <c r="C119" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f>IF(ISBLANK(B119),"",TEXT(B119, "dddd"))</f>
         <v>Tuesday</v>
       </c>
       <c r="D119" s="15"/>
@@ -4866,7 +5074,7 @@
         <v>46042</v>
       </c>
       <c r="C120" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f>IF(ISBLANK(B120),"",TEXT(B120, "dddd"))</f>
         <v>Tuesday</v>
       </c>
       <c r="D120" s="15"/>
@@ -4884,7 +5092,7 @@
         <v>46042</v>
       </c>
       <c r="C121" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f>IF(ISBLANK(B121),"",TEXT(B121, "dddd"))</f>
         <v>Tuesday</v>
       </c>
       <c r="D121" s="15"/>
@@ -4902,7 +5110,7 @@
         <v>46042</v>
       </c>
       <c r="C122" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f>IF(ISBLANK(B122),"",TEXT(B122, "dddd"))</f>
         <v>Tuesday</v>
       </c>
       <c r="D122" s="15"/>
@@ -4920,7 +5128,7 @@
         <v>46043</v>
       </c>
       <c r="C123" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f>IF(ISBLANK(B123),"",TEXT(B123, "dddd"))</f>
         <v>Wednesday</v>
       </c>
       <c r="D123" s="15"/>
@@ -4938,7 +5146,7 @@
         <v>46043</v>
       </c>
       <c r="C124" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f>IF(ISBLANK(B124),"",TEXT(B124, "dddd"))</f>
         <v>Wednesday</v>
       </c>
       <c r="D124" s="15"/>
@@ -4956,7 +5164,7 @@
         <v>46043</v>
       </c>
       <c r="C125" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f>IF(ISBLANK(B125),"",TEXT(B125, "dddd"))</f>
         <v>Wednesday</v>
       </c>
       <c r="D125" s="15"/>
@@ -4974,7 +5182,7 @@
         <v>46043</v>
       </c>
       <c r="C126" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f>IF(ISBLANK(B126),"",TEXT(B126, "dddd"))</f>
         <v>Wednesday</v>
       </c>
       <c r="D126" s="15"/>
@@ -4992,7 +5200,7 @@
         <v>46043</v>
       </c>
       <c r="C127" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f>IF(ISBLANK(B127),"",TEXT(B127, "dddd"))</f>
         <v>Wednesday</v>
       </c>
       <c r="D127" s="15"/>
@@ -5010,7 +5218,7 @@
         <v>46044</v>
       </c>
       <c r="C128" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f>IF(ISBLANK(B128),"",TEXT(B128, "dddd"))</f>
         <v>Thursday</v>
       </c>
       <c r="D128" s="15"/>
@@ -5028,7 +5236,7 @@
         <v>46044</v>
       </c>
       <c r="C129" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f>IF(ISBLANK(B129),"",TEXT(B129, "dddd"))</f>
         <v>Thursday</v>
       </c>
       <c r="D129" s="15"/>
@@ -5046,7 +5254,7 @@
         <v>46045</v>
       </c>
       <c r="C130" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f>IF(ISBLANK(B130),"",TEXT(B130, "dddd"))</f>
         <v>Friday</v>
       </c>
       <c r="D130" s="15"/>
@@ -5064,7 +5272,7 @@
         <v>46045</v>
       </c>
       <c r="C131" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f>IF(ISBLANK(B131),"",TEXT(B131, "dddd"))</f>
         <v>Friday</v>
       </c>
       <c r="D131" s="15"/>
@@ -5082,7 +5290,7 @@
         <v>46045</v>
       </c>
       <c r="C132" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f>IF(ISBLANK(B132),"",TEXT(B132, "dddd"))</f>
         <v>Friday</v>
       </c>
       <c r="D132" s="15"/>
@@ -5100,7 +5308,7 @@
         <v>46055</v>
       </c>
       <c r="C133" s="15" t="str">
-        <f t="shared" si="4"/>
+        <f>IF(ISBLANK(B133),"",TEXT(B133, "dddd"))</f>
         <v>Monday</v>
       </c>
       <c r="D133" s="15"/>
@@ -5114,141 +5322,185 @@
       <c r="H133" s="16"/>
     </row>
     <row r="134" spans="2:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="B134" s="13"/>
+      <c r="B134" s="13">
+        <v>46078</v>
+      </c>
       <c r="C134" s="15" t="str">
-        <f t="shared" si="4"/>
-        <v/>
+        <f>IF(ISBLANK(B134),"",TEXT(B134, "dddd"))</f>
+        <v>Wednesday</v>
       </c>
       <c r="D134" s="15"/>
       <c r="E134" s="74"/>
-      <c r="F134" s="15"/>
+      <c r="F134" s="15" t="s">
+        <v>291</v>
+      </c>
       <c r="G134" s="44"/>
       <c r="H134" s="16"/>
     </row>
-    <row r="135" spans="2:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="B135" s="13"/>
+    <row r="135" spans="2:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="B135" s="13">
+        <v>46079</v>
+      </c>
       <c r="C135" s="15" t="str">
-        <f t="shared" si="4"/>
-        <v/>
+        <f>IF(ISBLANK(B135),"",TEXT(B135, "dddd"))</f>
+        <v>Thursday</v>
       </c>
       <c r="D135" s="15"/>
       <c r="E135" s="74"/>
-      <c r="F135" s="15"/>
+      <c r="F135" s="15" t="s">
+        <v>295</v>
+      </c>
       <c r="G135" s="44"/>
       <c r="H135" s="16"/>
     </row>
-    <row r="136" spans="2:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="B136" s="13"/>
+    <row r="136" spans="2:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="B136" s="13">
+        <v>46079</v>
+      </c>
       <c r="C136" s="15" t="str">
-        <f t="shared" si="4"/>
-        <v/>
+        <f>IF(ISBLANK(B136),"",TEXT(B136, "dddd"))</f>
+        <v>Thursday</v>
       </c>
       <c r="D136" s="15"/>
       <c r="E136" s="74"/>
-      <c r="F136" s="15"/>
+      <c r="F136" s="11" t="s">
+        <v>298</v>
+      </c>
       <c r="G136" s="44"/>
       <c r="H136" s="16"/>
     </row>
     <row r="137" spans="2:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="B137" s="13"/>
+      <c r="B137" s="13">
+        <v>46079</v>
+      </c>
       <c r="C137" s="15" t="str">
-        <f t="shared" si="4"/>
-        <v/>
+        <f>IF(ISBLANK(B137),"",TEXT(B137, "dddd"))</f>
+        <v>Thursday</v>
       </c>
       <c r="D137" s="15"/>
       <c r="E137" s="74"/>
-      <c r="F137" s="15"/>
+      <c r="F137" s="15" t="s">
+        <v>299</v>
+      </c>
       <c r="G137" s="44"/>
       <c r="H137" s="16"/>
     </row>
     <row r="138" spans="2:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="B138" s="13"/>
+      <c r="B138" s="13">
+        <v>46080</v>
+      </c>
       <c r="C138" s="15" t="str">
-        <f t="shared" si="4"/>
-        <v/>
+        <f>IF(ISBLANK(B138),"",TEXT(B138, "dddd"))</f>
+        <v>Friday</v>
       </c>
       <c r="D138" s="15"/>
       <c r="E138" s="74"/>
-      <c r="F138" s="15"/>
+      <c r="F138" s="15" t="s">
+        <v>292</v>
+      </c>
       <c r="G138" s="44"/>
       <c r="H138" s="16"/>
     </row>
     <row r="139" spans="2:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="B139" s="13"/>
+      <c r="B139" s="13">
+        <v>46080</v>
+      </c>
       <c r="C139" s="15" t="str">
-        <f t="shared" si="4"/>
-        <v/>
+        <f>IF(ISBLANK(B139),"",TEXT(B139, "dddd"))</f>
+        <v>Friday</v>
       </c>
       <c r="D139" s="15"/>
       <c r="E139" s="74"/>
-      <c r="F139" s="15"/>
+      <c r="F139" s="15" t="s">
+        <v>300</v>
+      </c>
       <c r="G139" s="44"/>
       <c r="H139" s="16"/>
     </row>
     <row r="140" spans="2:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="B140" s="13"/>
+      <c r="B140" s="13">
+        <v>46080</v>
+      </c>
       <c r="C140" s="15" t="str">
-        <f t="shared" ref="C140:C171" si="5">IF(ISBLANK(B140),"",TEXT(B140, "dddd"))</f>
-        <v/>
+        <f>IF(ISBLANK(B140),"",TEXT(B140, "dddd"))</f>
+        <v>Friday</v>
       </c>
       <c r="D140" s="15"/>
       <c r="E140" s="74"/>
-      <c r="F140" s="15"/>
+      <c r="F140" s="80" t="s">
+        <v>290</v>
+      </c>
       <c r="G140" s="44"/>
       <c r="H140" s="16"/>
     </row>
-    <row r="141" spans="2:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="B141" s="13"/>
+    <row r="141" spans="2:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="B141" s="13">
+        <v>46080</v>
+      </c>
       <c r="C141" s="15" t="str">
-        <f t="shared" si="5"/>
-        <v/>
+        <f>IF(ISBLANK(B141),"",TEXT(B141, "dddd"))</f>
+        <v>Friday</v>
       </c>
       <c r="D141" s="15"/>
       <c r="E141" s="74"/>
-      <c r="F141" s="15"/>
+      <c r="F141" s="15" t="s">
+        <v>296</v>
+      </c>
       <c r="G141" s="44"/>
       <c r="H141" s="16"/>
     </row>
     <row r="142" spans="2:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="B142" s="13"/>
+      <c r="B142" s="13">
+        <v>46080</v>
+      </c>
       <c r="C142" s="15" t="str">
-        <f t="shared" si="5"/>
-        <v/>
+        <f>IF(ISBLANK(B142),"",TEXT(B142, "dddd"))</f>
+        <v>Friday</v>
       </c>
       <c r="D142" s="15"/>
       <c r="E142" s="74"/>
-      <c r="F142" s="15"/>
+      <c r="F142" s="15" t="s">
+        <v>297</v>
+      </c>
       <c r="G142" s="44"/>
       <c r="H142" s="16"/>
     </row>
     <row r="143" spans="2:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="B143" s="13"/>
+      <c r="B143" s="13">
+        <v>46083</v>
+      </c>
       <c r="C143" s="15" t="str">
-        <f t="shared" si="5"/>
-        <v/>
+        <f>IF(ISBLANK(B143),"",TEXT(B143, "dddd"))</f>
+        <v>Monday</v>
       </c>
       <c r="D143" s="15"/>
       <c r="E143" s="74"/>
-      <c r="F143" s="15"/>
+      <c r="F143" s="15" t="s">
+        <v>293</v>
+      </c>
       <c r="G143" s="44"/>
       <c r="H143" s="16"/>
     </row>
-    <row r="144" spans="2:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="B144" s="13"/>
+    <row r="144" spans="2:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="B144" s="13">
+        <v>46083</v>
+      </c>
       <c r="C144" s="15" t="str">
-        <f t="shared" si="5"/>
-        <v/>
+        <f>IF(ISBLANK(B144),"",TEXT(B144, "dddd"))</f>
+        <v>Monday</v>
       </c>
       <c r="D144" s="15"/>
       <c r="E144" s="74"/>
-      <c r="F144" s="15"/>
+      <c r="F144" s="15" t="s">
+        <v>294</v>
+      </c>
       <c r="G144" s="44"/>
       <c r="H144" s="16"/>
     </row>
     <row r="145" spans="2:8" ht="16" x14ac:dyDescent="0.2">
       <c r="B145" s="13"/>
       <c r="C145" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f>IF(ISBLANK(B145),"",TEXT(B145, "dddd"))</f>
         <v/>
       </c>
       <c r="D145" s="15"/>
@@ -5260,7 +5512,7 @@
     <row r="146" spans="2:8" ht="16" x14ac:dyDescent="0.2">
       <c r="B146" s="13"/>
       <c r="C146" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f>IF(ISBLANK(B146),"",TEXT(B146, "dddd"))</f>
         <v/>
       </c>
       <c r="D146" s="15"/>
@@ -5272,19 +5524,19 @@
     <row r="147" spans="2:8" ht="16" x14ac:dyDescent="0.2">
       <c r="B147" s="13"/>
       <c r="C147" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f>IF(ISBLANK(B147),"",TEXT(B147, "dddd"))</f>
         <v/>
       </c>
       <c r="D147" s="15"/>
       <c r="E147" s="74"/>
-      <c r="F147" s="15"/>
+      <c r="F147" s="11"/>
       <c r="G147" s="44"/>
       <c r="H147" s="16"/>
     </row>
     <row r="148" spans="2:8" ht="16" x14ac:dyDescent="0.2">
       <c r="B148" s="13"/>
       <c r="C148" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f>IF(ISBLANK(B148),"",TEXT(B148, "dddd"))</f>
         <v/>
       </c>
       <c r="D148" s="15"/>
@@ -5296,285 +5548,267 @@
     <row r="149" spans="2:8" ht="16" x14ac:dyDescent="0.2">
       <c r="B149" s="13"/>
       <c r="C149" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f>IF(ISBLANK(B149),"",TEXT(B149, "dddd"))</f>
         <v/>
       </c>
       <c r="D149" s="15"/>
       <c r="E149" s="74"/>
-      <c r="F149" s="15" t="s">
-        <v>182</v>
-      </c>
-      <c r="G149" s="44" t="s">
-        <v>227</v>
-      </c>
+      <c r="F149" s="15"/>
+      <c r="G149" s="44"/>
       <c r="H149" s="16"/>
     </row>
-    <row r="150" spans="2:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="150" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B150" s="13"/>
-      <c r="C150" s="15" t="str">
-        <f t="shared" si="5"/>
-        <v/>
-      </c>
+      <c r="C150" s="15"/>
       <c r="D150" s="15"/>
       <c r="E150" s="74"/>
       <c r="F150" s="15"/>
-      <c r="G150" s="44" t="s">
-        <v>231</v>
-      </c>
+      <c r="G150" s="44"/>
       <c r="H150" s="16"/>
     </row>
-    <row r="151" spans="2:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="151" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B151" s="13"/>
-      <c r="C151" s="15" t="str">
-        <f t="shared" si="5"/>
-        <v/>
-      </c>
+      <c r="C151" s="15"/>
       <c r="D151" s="15"/>
       <c r="E151" s="74"/>
       <c r="F151" s="15"/>
-      <c r="G151" s="44" t="s">
-        <v>229</v>
-      </c>
+      <c r="G151" s="44"/>
       <c r="H151" s="16"/>
     </row>
-    <row r="152" spans="2:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="152" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B152" s="13"/>
-      <c r="C152" s="15" t="str">
-        <f t="shared" si="5"/>
-        <v/>
-      </c>
+      <c r="C152" s="15"/>
       <c r="D152" s="15"/>
       <c r="E152" s="74"/>
-      <c r="F152" s="15" t="s">
-        <v>226</v>
-      </c>
-      <c r="G152" s="44" t="s">
-        <v>230</v>
-      </c>
+      <c r="F152" s="15"/>
+      <c r="G152" s="44"/>
       <c r="H152" s="16"/>
     </row>
-    <row r="153" spans="2:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="153" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B153" s="13"/>
-      <c r="C153" s="15" t="str">
-        <f t="shared" si="5"/>
-        <v/>
-      </c>
+      <c r="C153" s="15"/>
       <c r="D153" s="15"/>
       <c r="E153" s="74"/>
-      <c r="F153" s="15" t="s">
-        <v>178</v>
-      </c>
-      <c r="G153" s="44" t="s">
-        <v>140</v>
-      </c>
+      <c r="F153" s="15"/>
+      <c r="G153" s="44"/>
       <c r="H153" s="16"/>
     </row>
-    <row r="154" spans="2:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="154" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B154" s="13"/>
-      <c r="C154" s="15" t="str">
-        <f t="shared" si="5"/>
-        <v/>
-      </c>
+      <c r="C154" s="15"/>
       <c r="D154" s="15"/>
       <c r="E154" s="74"/>
-      <c r="F154" s="15" t="s">
-        <v>181</v>
-      </c>
-      <c r="G154" s="44" t="s">
-        <v>140</v>
-      </c>
+      <c r="F154" s="15"/>
+      <c r="G154" s="44"/>
       <c r="H154" s="16"/>
     </row>
     <row r="155" spans="2:8" ht="16" x14ac:dyDescent="0.2">
       <c r="B155" s="13"/>
       <c r="C155" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f>IF(ISBLANK(B155),"",TEXT(B155, "dddd"))</f>
         <v/>
       </c>
       <c r="D155" s="15"/>
       <c r="E155" s="74"/>
-      <c r="F155" s="15" t="s">
-        <v>169</v>
-      </c>
-      <c r="G155" s="44" t="s">
-        <v>228</v>
-      </c>
+      <c r="F155" s="15"/>
+      <c r="G155" s="44"/>
       <c r="H155" s="16"/>
     </row>
     <row r="156" spans="2:8" ht="16" x14ac:dyDescent="0.2">
       <c r="B156" s="13"/>
       <c r="C156" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f>IF(ISBLANK(B156),"",TEXT(B156, "dddd"))</f>
         <v/>
       </c>
       <c r="D156" s="15"/>
-      <c r="E156" s="44"/>
+      <c r="E156" s="74"/>
       <c r="F156" s="15" t="s">
-        <v>222</v>
+        <v>182</v>
       </c>
       <c r="G156" s="44" t="s">
-        <v>140</v>
-      </c>
-      <c r="H156" s="17"/>
+        <v>227</v>
+      </c>
+      <c r="H156" s="16"/>
     </row>
     <row r="157" spans="2:8" ht="16" x14ac:dyDescent="0.2">
       <c r="B157" s="13"/>
       <c r="C157" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f>IF(ISBLANK(B157),"",TEXT(B157, "dddd"))</f>
         <v/>
       </c>
       <c r="D157" s="15"/>
-      <c r="E157" s="44"/>
-      <c r="F157" s="15" t="s">
-        <v>223</v>
-      </c>
+      <c r="E157" s="74"/>
+      <c r="F157" s="15"/>
       <c r="G157" s="44" t="s">
-        <v>140</v>
-      </c>
-      <c r="H157" s="17"/>
+        <v>231</v>
+      </c>
+      <c r="H157" s="16"/>
     </row>
     <row r="158" spans="2:8" ht="16" x14ac:dyDescent="0.2">
       <c r="B158" s="13"/>
       <c r="C158" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f>IF(ISBLANK(B158),"",TEXT(B158, "dddd"))</f>
         <v/>
       </c>
       <c r="D158" s="15"/>
       <c r="E158" s="74"/>
-      <c r="F158" s="15" t="s">
-        <v>233</v>
-      </c>
-      <c r="G158" s="44"/>
+      <c r="F158" s="15"/>
+      <c r="G158" s="44" t="s">
+        <v>229</v>
+      </c>
       <c r="H158" s="16"/>
     </row>
     <row r="159" spans="2:8" ht="16" x14ac:dyDescent="0.2">
       <c r="B159" s="13"/>
       <c r="C159" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f>IF(ISBLANK(B159),"",TEXT(B159, "dddd"))</f>
         <v/>
       </c>
       <c r="D159" s="15"/>
       <c r="E159" s="74"/>
       <c r="F159" s="15" t="s">
-        <v>244</v>
-      </c>
-      <c r="G159" s="44"/>
+        <v>226</v>
+      </c>
+      <c r="G159" s="44" t="s">
+        <v>230</v>
+      </c>
       <c r="H159" s="16"/>
     </row>
     <row r="160" spans="2:8" ht="16" x14ac:dyDescent="0.2">
       <c r="B160" s="13"/>
       <c r="C160" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f>IF(ISBLANK(B160),"",TEXT(B160, "dddd"))</f>
         <v/>
       </c>
       <c r="D160" s="15"/>
       <c r="E160" s="74"/>
       <c r="F160" s="15" t="s">
-        <v>245</v>
-      </c>
-      <c r="G160" s="44"/>
+        <v>178</v>
+      </c>
+      <c r="G160" s="44" t="s">
+        <v>140</v>
+      </c>
       <c r="H160" s="16"/>
     </row>
     <row r="161" spans="2:8" ht="16" x14ac:dyDescent="0.2">
       <c r="B161" s="13"/>
       <c r="C161" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f>IF(ISBLANK(B161),"",TEXT(B161, "dddd"))</f>
         <v/>
       </c>
       <c r="D161" s="15"/>
       <c r="E161" s="74"/>
       <c r="F161" s="15" t="s">
-        <v>246</v>
-      </c>
-      <c r="G161" s="44"/>
+        <v>181</v>
+      </c>
+      <c r="G161" s="44" t="s">
+        <v>140</v>
+      </c>
       <c r="H161" s="16"/>
     </row>
     <row r="162" spans="2:8" ht="16" x14ac:dyDescent="0.2">
       <c r="B162" s="13"/>
       <c r="C162" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f>IF(ISBLANK(B162),"",TEXT(B162, "dddd"))</f>
         <v/>
       </c>
       <c r="D162" s="15"/>
       <c r="E162" s="74"/>
       <c r="F162" s="15" t="s">
-        <v>247</v>
-      </c>
-      <c r="G162" s="44"/>
+        <v>169</v>
+      </c>
+      <c r="G162" s="44" t="s">
+        <v>228</v>
+      </c>
       <c r="H162" s="16"/>
     </row>
     <row r="163" spans="2:8" ht="16" x14ac:dyDescent="0.2">
       <c r="B163" s="13"/>
       <c r="C163" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f>IF(ISBLANK(B163),"",TEXT(B163, "dddd"))</f>
         <v/>
       </c>
       <c r="D163" s="15"/>
-      <c r="E163" s="74"/>
+      <c r="E163" s="44"/>
       <c r="F163" s="15" t="s">
-        <v>248</v>
-      </c>
-      <c r="G163" s="44"/>
-      <c r="H163" s="16"/>
+        <v>222</v>
+      </c>
+      <c r="G163" s="44" t="s">
+        <v>140</v>
+      </c>
+      <c r="H163" s="17"/>
     </row>
     <row r="164" spans="2:8" ht="16" x14ac:dyDescent="0.2">
       <c r="B164" s="13"/>
       <c r="C164" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f>IF(ISBLANK(B164),"",TEXT(B164, "dddd"))</f>
         <v/>
       </c>
       <c r="D164" s="15"/>
-      <c r="E164" s="74"/>
-      <c r="F164" s="11" t="s">
-        <v>249</v>
-      </c>
-      <c r="G164" s="44"/>
-      <c r="H164" s="16"/>
+      <c r="E164" s="44"/>
+      <c r="F164" s="15" t="s">
+        <v>223</v>
+      </c>
+      <c r="G164" s="44" t="s">
+        <v>140</v>
+      </c>
+      <c r="H164" s="17"/>
     </row>
     <row r="165" spans="2:8" ht="16" x14ac:dyDescent="0.2">
       <c r="B165" s="13"/>
       <c r="C165" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f>IF(ISBLANK(B165),"",TEXT(B165, "dddd"))</f>
         <v/>
       </c>
       <c r="D165" s="15"/>
       <c r="E165" s="74"/>
-      <c r="F165" s="15"/>
+      <c r="F165" s="15" t="s">
+        <v>233</v>
+      </c>
       <c r="G165" s="44"/>
       <c r="H165" s="16"/>
     </row>
     <row r="166" spans="2:8" ht="16" x14ac:dyDescent="0.2">
       <c r="B166" s="13"/>
       <c r="C166" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f>IF(ISBLANK(B166),"",TEXT(B166, "dddd"))</f>
         <v/>
       </c>
       <c r="D166" s="15"/>
-      <c r="E166" s="44"/>
-      <c r="F166" s="15"/>
+      <c r="E166" s="74"/>
+      <c r="F166" s="15" t="s">
+        <v>244</v>
+      </c>
       <c r="G166" s="44"/>
-      <c r="H166" s="17"/>
+      <c r="H166" s="16"/>
     </row>
     <row r="167" spans="2:8" ht="16" x14ac:dyDescent="0.2">
       <c r="B167" s="13"/>
       <c r="C167" s="15" t="str">
-        <f t="shared" si="5"/>
+        <f>IF(ISBLANK(B167),"",TEXT(B167, "dddd"))</f>
         <v/>
       </c>
       <c r="D167" s="15"/>
-      <c r="E167" s="44"/>
-      <c r="F167" s="15"/>
+      <c r="E167" s="74"/>
+      <c r="F167" s="15" t="s">
+        <v>245</v>
+      </c>
       <c r="G167" s="44"/>
-      <c r="H167" s="17"/>
-    </row>
-    <row r="168" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="H167" s="16"/>
+    </row>
+    <row r="168" spans="2:8" ht="16" x14ac:dyDescent="0.2">
       <c r="B168" s="13"/>
-      <c r="C168" s="15"/>
+      <c r="C168" s="15" t="str">
+        <f>IF(ISBLANK(B168),"",TEXT(B168, "dddd"))</f>
+        <v/>
+      </c>
       <c r="D168" s="15"/>
-      <c r="E168" s="44"/>
-      <c r="F168" s="15"/>
+      <c r="E168" s="74"/>
+      <c r="F168" s="15" t="s">
+        <v>246</v>
+      </c>
       <c r="G168" s="44"/>
-      <c r="H168" s="17"/>
+      <c r="H168" s="16"/>
     </row>
     <row r="169" spans="2:8" ht="16" x14ac:dyDescent="0.2">
       <c r="B169" s="13"/>
@@ -5583,10 +5817,12 @@
         <v/>
       </c>
       <c r="D169" s="15"/>
-      <c r="E169" s="44"/>
-      <c r="F169" s="15"/>
+      <c r="E169" s="74"/>
+      <c r="F169" s="15" t="s">
+        <v>247</v>
+      </c>
       <c r="G169" s="44"/>
-      <c r="H169" s="17"/>
+      <c r="H169" s="16"/>
     </row>
     <row r="170" spans="2:8" ht="16" x14ac:dyDescent="0.2">
       <c r="B170" s="13"/>
@@ -5595,10 +5831,12 @@
         <v/>
       </c>
       <c r="D170" s="15"/>
-      <c r="E170" s="44"/>
-      <c r="F170" s="15"/>
+      <c r="E170" s="74"/>
+      <c r="F170" s="15" t="s">
+        <v>248</v>
+      </c>
       <c r="G170" s="44"/>
-      <c r="H170" s="17"/>
+      <c r="H170" s="16"/>
     </row>
     <row r="171" spans="2:8" ht="16" x14ac:dyDescent="0.2">
       <c r="B171" s="13"/>
@@ -5607,44 +5845,131 @@
         <v/>
       </c>
       <c r="D171" s="15"/>
-      <c r="E171" s="44"/>
-      <c r="F171" s="15"/>
+      <c r="E171" s="74"/>
+      <c r="F171" s="11" t="s">
+        <v>249</v>
+      </c>
       <c r="G171" s="44"/>
-      <c r="H171" s="17"/>
-    </row>
-    <row r="172" spans="2:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B172" s="46"/>
-      <c r="C172" s="18"/>
-      <c r="D172" s="18"/>
-      <c r="E172" s="45"/>
-      <c r="F172" s="18"/>
-      <c r="G172" s="45"/>
-      <c r="H172" s="19"/>
+      <c r="H171" s="16"/>
+    </row>
+    <row r="172" spans="2:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="B172" s="13"/>
+      <c r="C172" s="15" t="str">
+        <f>IF(ISBLANK(B172),"",TEXT(B172, "dddd"))</f>
+        <v/>
+      </c>
+      <c r="D172" s="15"/>
+      <c r="E172" s="74"/>
+      <c r="F172" s="15"/>
+      <c r="G172" s="44"/>
+      <c r="H172" s="16"/>
+    </row>
+    <row r="173" spans="2:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="B173" s="13"/>
+      <c r="C173" s="15" t="str">
+        <f>IF(ISBLANK(B173),"",TEXT(B173, "dddd"))</f>
+        <v/>
+      </c>
+      <c r="D173" s="15"/>
+      <c r="E173" s="44"/>
+      <c r="F173" s="15"/>
+      <c r="G173" s="44"/>
+      <c r="H173" s="17"/>
+    </row>
+    <row r="174" spans="2:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="B174" s="13"/>
+      <c r="C174" s="15" t="str">
+        <f>IF(ISBLANK(B174),"",TEXT(B174, "dddd"))</f>
+        <v/>
+      </c>
+      <c r="D174" s="15"/>
+      <c r="E174" s="44"/>
+      <c r="F174" s="15"/>
+      <c r="G174" s="44"/>
+      <c r="H174" s="17"/>
+    </row>
+    <row r="175" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B175" s="13"/>
+      <c r="C175" s="15"/>
+      <c r="D175" s="15"/>
+      <c r="E175" s="44"/>
+      <c r="F175" s="15"/>
+      <c r="G175" s="44"/>
+      <c r="H175" s="17"/>
+    </row>
+    <row r="176" spans="2:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="B176" s="13"/>
+      <c r="C176" s="15" t="str">
+        <f>IF(ISBLANK(B176),"",TEXT(B176, "dddd"))</f>
+        <v/>
+      </c>
+      <c r="D176" s="15"/>
+      <c r="E176" s="44"/>
+      <c r="F176" s="15"/>
+      <c r="G176" s="44"/>
+      <c r="H176" s="17"/>
+    </row>
+    <row r="177" spans="2:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="B177" s="13"/>
+      <c r="C177" s="15" t="str">
+        <f>IF(ISBLANK(B177),"",TEXT(B177, "dddd"))</f>
+        <v/>
+      </c>
+      <c r="D177" s="15"/>
+      <c r="E177" s="44"/>
+      <c r="F177" s="15"/>
+      <c r="G177" s="44"/>
+      <c r="H177" s="17"/>
+    </row>
+    <row r="178" spans="2:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="B178" s="13"/>
+      <c r="C178" s="15" t="str">
+        <f>IF(ISBLANK(B178),"",TEXT(B178, "dddd"))</f>
+        <v/>
+      </c>
+      <c r="D178" s="15"/>
+      <c r="E178" s="44"/>
+      <c r="F178" s="15"/>
+      <c r="G178" s="44"/>
+      <c r="H178" s="17"/>
+    </row>
+    <row r="179" spans="2:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B179" s="46"/>
+      <c r="C179" s="18"/>
+      <c r="D179" s="18"/>
+      <c r="E179" s="45"/>
+      <c r="F179" s="18"/>
+      <c r="G179" s="45"/>
+      <c r="H179" s="19"/>
     </row>
   </sheetData>
-  <autoFilter ref="B2:H172" xr:uid="{40A518F1-E8D1-4EDA-B8FC-EAEFD9F39116}"/>
-  <conditionalFormatting sqref="B2:H457">
-    <cfRule type="expression" dxfId="12" priority="7">
+  <autoFilter ref="B2:H179" xr:uid="{40A518F1-E8D1-4EDA-B8FC-EAEFD9F39116}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:H179">
+      <sortCondition ref="B2:B179"/>
+    </sortState>
+  </autoFilter>
+  <conditionalFormatting sqref="B2:H500">
+    <cfRule type="expression" dxfId="12" priority="7" stopIfTrue="1">
       <formula>$C2=Saturday</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="11" priority="8">
+    <cfRule type="expression" dxfId="14" priority="8">
       <formula>$C2="Monday"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="9">
+    <cfRule type="expression" dxfId="17" priority="9">
       <formula>$C2="Tuesday"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="10">
+    <cfRule type="expression" dxfId="16" priority="10" stopIfTrue="1">
       <formula>$C2="Wednesday"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="11">
+    <cfRule type="expression" dxfId="15" priority="11">
       <formula>$C2="Thursday"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="12">
+    <cfRule type="expression" dxfId="13" priority="12">
       <formula>$C2="Friday"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E33:E172 H33:H172" xr:uid="{F96E5036-0CE7-4348-B733-74DDF2C8E069}">
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E33:E179 H33:H179" xr:uid="{F96E5036-0CE7-4348-B733-74DDF2C8E069}">
       <formula1>45658</formula1>
       <formula2>46388</formula2>
     </dataValidation>
@@ -5702,6 +6027,9 @@
       </c>
       <c r="C3">
         <v>142</v>
+      </c>
+      <c r="I3">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -6508,25 +6836,25 @@
     <mergeCell ref="B2:N2"/>
   </mergeCells>
   <conditionalFormatting sqref="B4:N28">
-    <cfRule type="expression" dxfId="6" priority="1">
+    <cfRule type="expression" dxfId="36" priority="1">
       <formula>LEFT($B4,1)="7"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="2">
+    <cfRule type="expression" dxfId="35" priority="2">
       <formula>LEFT($B4,1)="1"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="3">
+    <cfRule type="expression" dxfId="34" priority="3">
       <formula>LEFT($B4,1)="2"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="4">
+    <cfRule type="expression" dxfId="33" priority="4">
       <formula>LEFT($B4,1)="3"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="5">
+    <cfRule type="expression" dxfId="32" priority="5">
       <formula>LEFT($B4,1)="4"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="6">
+    <cfRule type="expression" dxfId="31" priority="6">
       <formula>LEFT($B4,1)="5"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="7">
+    <cfRule type="expression" dxfId="30" priority="7">
       <formula>LEFT($B4,1)="6"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>